<commit_message>
Added new projectors to KB0003
</commit_message>
<xml_diff>
--- a/knowledgebase.xlsx
+++ b/knowledgebase.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76CB8B1B-971C-F04A-ADF2-F3B8687BD02E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D21DB9B7-6722-3A4E-8A56-337DAF510C1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1840" yWindow="1660" windowWidth="17740" windowHeight="14320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1840" yWindow="1660" windowWidth="17740" windowHeight="13660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Issues" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="446">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="447">
   <si>
     <t xml:space="preserve"> IssueID </t>
   </si>
@@ -1501,6 +1501,9 @@
   </si>
   <si>
     <t>#propresenter, #network</t>
+  </si>
+  <si>
+    <t>ZVVU-A001, ZVVU-A002, ZVVU-A003, 2604-2403,2604-2402,2604-2401</t>
   </si>
 </sst>
 </file>
@@ -2159,7 +2162,7 @@
         <v>28</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>29</v>
+        <v>446</v>
       </c>
       <c r="K5" s="1" t="s">
         <v>46</v>

</xml_diff>

<commit_message>
added KB item for finicky vs88
</commit_message>
<xml_diff>
--- a/knowledgebase.xlsx
+++ b/knowledgebase.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A654F2F-ED3C-7144-B57C-3DC9BE5D4E05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{084B132C-49AB-1A4E-9FC8-C28BC62B3282}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="609" uniqueCount="471">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="476">
   <si>
     <t xml:space="preserve"> IssueID </t>
   </si>
@@ -1577,12 +1577,27 @@
   <si>
     <t>May need to check both ends of cable</t>
   </si>
+  <si>
+    <t>KB0042</t>
+  </si>
+  <si>
+    <t>VS88 Video Matrix unresponsive to newtork</t>
+  </si>
+  <si>
+    <t>Does not repsond to network ping</t>
+  </si>
+  <si>
+    <t>Monitoring of network status if Kramer VS88DT video matrix, it doesn't respond to Ping</t>
+  </si>
+  <si>
+    <t>Physical device changes can confuse this device requiring a reboot.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1603,6 +1618,13 @@
       <name val="Menlo"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1612,7 +1634,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -1620,11 +1642,48 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF47D359"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF47D359"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF47D359"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF47D359"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF47D359"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF47D359"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF47D359"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF47D359"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1636,6 +1695,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1707,27 +1775,27 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8DA13CB4-8680-0D4C-A016-6564C2E20834}" name="Table1" displayName="Table1" ref="A1:O43" totalsRowShown="0" headerRowDxfId="16" dataDxfId="0">
-  <autoFilter ref="A1:O43" xr:uid="{8DA13CB4-8680-0D4C-A016-6564C2E20834}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8DA13CB4-8680-0D4C-A016-6564C2E20834}" name="Table1" displayName="Table1" ref="A1:O44" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
+  <autoFilter ref="A1:O44" xr:uid="{8DA13CB4-8680-0D4C-A016-6564C2E20834}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:O41">
     <sortCondition ref="A2:A41"/>
   </sortState>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{F5D9425D-17E4-814F-893B-3266F2DAF7F0}" name=" IssueID " dataDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{99B6ADBC-8781-B846-821D-0367B521DD89}" name=" Category " dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{B6DBC451-2B1C-F94A-A01B-8135E89CBAC8}" name=" Subcategory " dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{FB7DD802-E795-B047-BE37-D8BB7C6A5BAD}" name=" Title " dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{07201179-6B39-8949-844B-CEE11E6EDB49}" name=" Symptom " dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{0485B2F9-34C2-CA48-AB6F-0BC3BA51FBC0}" name=" TriggerConditions " dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{4183B9DE-D94A-BD4A-8F0E-B7A760717C5F}" name=" LikelyCause " dataDxfId="9"/>
-    <tableColumn id="8" xr3:uid="{62C265AB-4FCB-1046-AF2C-3C97D014F136}" name=" RecoverySteps " dataDxfId="8"/>
-    <tableColumn id="9" xr3:uid="{5A36F6EB-E991-8D4D-94E7-05C8CA75197F}" name=" AppliesToAssetType " dataDxfId="7"/>
-    <tableColumn id="10" xr3:uid="{9AEAF97E-3F51-A043-A89E-F8F005226CB6}" name="AppliesToAssetTag" dataDxfId="6"/>
-    <tableColumn id="11" xr3:uid="{5C0A625C-1C65-5A4A-AF4C-D0F44F2906A2}" name=" Tags " dataDxfId="5"/>
-    <tableColumn id="12" xr3:uid="{7FF7E833-E899-C24E-8BBE-767CE59AEB38}" name="SeeAlso" dataDxfId="4"/>
-    <tableColumn id="13" xr3:uid="{E3A9225A-7773-DA40-A1EE-0FBB1F1DFED4}" name=" SortOrder " dataDxfId="3"/>
-    <tableColumn id="14" xr3:uid="{013C7458-C36D-8340-BDE2-1630AA3F099E}" name=" Active " dataDxfId="2"/>
-    <tableColumn id="15" xr3:uid="{03B11681-0EC6-4C43-8C60-99EAC922882E}" name=" Notes " dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{F5D9425D-17E4-814F-893B-3266F2DAF7F0}" name=" IssueID " dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{99B6ADBC-8781-B846-821D-0367B521DD89}" name=" Category " dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{B6DBC451-2B1C-F94A-A01B-8135E89CBAC8}" name=" Subcategory " dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{FB7DD802-E795-B047-BE37-D8BB7C6A5BAD}" name=" Title " dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{07201179-6B39-8949-844B-CEE11E6EDB49}" name=" Symptom " dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{0485B2F9-34C2-CA48-AB6F-0BC3BA51FBC0}" name=" TriggerConditions " dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{4183B9DE-D94A-BD4A-8F0E-B7A760717C5F}" name=" LikelyCause " dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{62C265AB-4FCB-1046-AF2C-3C97D014F136}" name=" RecoverySteps " dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{5A36F6EB-E991-8D4D-94E7-05C8CA75197F}" name=" AppliesToAssetType " dataDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{9AEAF97E-3F51-A043-A89E-F8F005226CB6}" name="AppliesToAssetTag" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{5C0A625C-1C65-5A4A-AF4C-D0F44F2906A2}" name=" Tags " dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{7FF7E833-E899-C24E-8BBE-767CE59AEB38}" name="SeeAlso" dataDxfId="3"/>
+    <tableColumn id="13" xr3:uid="{E3A9225A-7773-DA40-A1EE-0FBB1F1DFED4}" name=" SortOrder " dataDxfId="2"/>
+    <tableColumn id="14" xr3:uid="{013C7458-C36D-8340-BDE2-1630AA3F099E}" name=" Active " dataDxfId="1"/>
+    <tableColumn id="15" xr3:uid="{03B11681-0EC6-4C43-8C60-99EAC922882E}" name=" Notes " dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2050,7 +2118,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O43"/>
+  <dimension ref="A1:O44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.5" style="1" customWidth="1"/>
@@ -2781,7 +2849,9 @@
       <c r="K17" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="L17" s="4"/>
+      <c r="L17" s="6" t="s">
+        <v>471</v>
+      </c>
       <c r="M17" s="4">
         <v>16</v>
       </c>
@@ -3900,6 +3970,53 @@
       </c>
       <c r="O43" s="4" t="s">
         <v>470</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" ht="51" x14ac:dyDescent="0.2">
+      <c r="A44" s="6" t="s">
+        <v>471</v>
+      </c>
+      <c r="B44" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C44" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="D44" s="7" t="s">
+        <v>472</v>
+      </c>
+      <c r="E44" s="7" t="s">
+        <v>473</v>
+      </c>
+      <c r="F44" s="7" t="s">
+        <v>474</v>
+      </c>
+      <c r="G44" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="H44" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="I44" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="J44" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="K44" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="L44" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="M44" s="7">
+        <v>44</v>
+      </c>
+      <c r="N44" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="O44" s="8" t="s">
+        <v>475</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adding issue for keyboard
</commit_message>
<xml_diff>
--- a/knowledgebase.xlsx
+++ b/knowledgebase.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{084B132C-49AB-1A4E-9FC8-C28BC62B3282}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7007EA63-CFA4-DE42-8677-BE15FBF440E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="476">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="637" uniqueCount="484">
   <si>
     <t xml:space="preserve"> IssueID </t>
   </si>
@@ -1591,6 +1591,30 @@
   </si>
   <si>
     <t>Physical device changes can confuse this device requiring a reboot.</t>
+  </si>
+  <si>
+    <t>KB0043</t>
+  </si>
+  <si>
+    <t>Keyboard stops working</t>
+  </si>
+  <si>
+    <t>When trying to operate Propresenter, the keyboard stops working</t>
+  </si>
+  <si>
+    <t>Seems to be a random event</t>
+  </si>
+  <si>
+    <t>Keyboard lost USB connection to the KVM unit.</t>
+  </si>
+  <si>
+    <t>unplug and replug the keyboard</t>
+  </si>
+  <si>
+    <t>CUMU-G002, 2603-1105</t>
+  </si>
+  <si>
+    <t>#propresenter, #keyboard</t>
   </si>
 </sst>
 </file>
@@ -1775,8 +1799,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8DA13CB4-8680-0D4C-A016-6564C2E20834}" name="Table1" displayName="Table1" ref="A1:O44" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
-  <autoFilter ref="A1:O44" xr:uid="{8DA13CB4-8680-0D4C-A016-6564C2E20834}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8DA13CB4-8680-0D4C-A016-6564C2E20834}" name="Table1" displayName="Table1" ref="A1:O45" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
+  <autoFilter ref="A1:O45" xr:uid="{8DA13CB4-8680-0D4C-A016-6564C2E20834}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:O41">
     <sortCondition ref="A2:A41"/>
   </sortState>
@@ -2118,7 +2142,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O44"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.5" style="1" customWidth="1"/>
@@ -4018,6 +4042,51 @@
       <c r="O44" s="8" t="s">
         <v>475</v>
       </c>
+    </row>
+    <row r="45" spans="1:15" ht="51" x14ac:dyDescent="0.2">
+      <c r="A45" s="4" t="s">
+        <v>476</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>477</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>479</v>
+      </c>
+      <c r="G45" s="4" t="s">
+        <v>480</v>
+      </c>
+      <c r="H45" s="4" t="s">
+        <v>481</v>
+      </c>
+      <c r="I45" s="4" t="s">
+        <v>317</v>
+      </c>
+      <c r="J45" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="K45" s="4" t="s">
+        <v>483</v>
+      </c>
+      <c r="L45" s="4" t="s">
+        <v>455</v>
+      </c>
+      <c r="M45" s="4">
+        <v>45</v>
+      </c>
+      <c r="N45" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="O45" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
cleaned excessive line breaks
</commit_message>
<xml_diff>
--- a/knowledgebase.xlsx
+++ b/knowledgebase.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC828064-3D63-644C-AC6A-83D16148653F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8561E90-EC21-6940-9F25-D987D6FFA522}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -171,9 +171,6 @@
     <t>Intermittent network connectivity issues between the control device, the network infrastructure, and the projector's internal web server, or the projector's network interface has frozen.</t>
   </si>
   <si>
-    <t>You need to be pretty much directly below each projection screen and point the remote at the projector. One remote will do all three but you will have to change the selector switch for each projector (not sure if the switch is labelled 1,2,3 or A,B,C.) The east screen is the "first" ( A or 1).</t>
-  </si>
-  <si>
     <t>#video, #projector, #network</t>
   </si>
   <si>
@@ -205,14 +202,6 @@
   </si>
   <si>
     <t>OBS software on CUMU-G001 displays a black screen or 'No Signal' message for the input from the Web Presenter, even though the Web Presenter itself shows an active video signal on its own display.</t>
-  </si>
-  <si>
-    <t>Occurs sporadically after system startup, or if the Web Presenter's USB connection to the computer (CUMU-G001) is
-         disturbed.</t>
-  </si>
-  <si>
-    <t>The USB driver for the Web Presenter on CUMU-G001 has become unresponsive, or the USB connection has momentarily dropped,
-         requiring a reset of the USB device to re-establish communication.</t>
   </si>
   <si>
     <t>Pull the plug and reinsert on the USB cable going into to the computer (CUMU-G001). The cable has a label "Web Camera"</t>
@@ -257,18 +246,6 @@
     <t>ProPresenter Lyric Overlay Not Appearing on ATEM</t>
   </si>
   <si>
-    <t>Upon activating the 'Key 1 Cut' in ATEM Software Control or pressing the 'Lyrics' button on the Stream Deck, the ProPresenter lyric
-         overlay fails to appear on the program output.</t>
-  </si>
-  <si>
-    <t>Observed when attempting to display lyric overlays after an ATEM software update, system reconfiguration, or if keyer
-         settings were manually adjusted.</t>
-  </si>
-  <si>
-    <t>Incorrect or altered 'Key 1' DSK (Downstream Keyer) settings within the ATEM software, specifically the 'Fill Source', 'Key
-         Source', or 'Key Type' parameters, preventing the overlay from rendering correctly.</t>
-  </si>
-  <si>
     <t>Return the key settings to correct values, running macro 1 is the easiest way to do so.</t>
   </si>
   <si>
@@ -290,17 +267,9 @@
     <t>Blackout Blind Detached from Side Track</t>
   </si>
   <si>
-    <t>A motorized blackout blind is visibly out of its side track, causing it to be stuck during movement or fail to fully seal against the
-         window frame.</t>
-  </si>
-  <si>
     <t>May occur during normal operation (raising or lowering the blind), or if the blind encounters an obstruction.</t>
   </si>
   <si>
-    <t>Misalignment or obstruction within the blind's track system, excessive tension on the fabric, or a mechanical issue with the
-         motor or winding mechanism causing it to dislodge.</t>
-  </si>
-  <si>
     <t>Running the blinds up and down a **little** bit at a time can sometimes get them back in their track. An assistant at the blind can reach in behind and help guide them in. If it is more than a few inches, a ladder may be required to reinsert the blind into the track.</t>
   </si>
   <si>
@@ -317,10 +286,6 @@
   </si>
   <si>
     <t>Adjusting faders or pressing playback buttons on the lighting console fails to alter the light levels or trigger programmed cues.</t>
-  </si>
-  <si>
-    <t>Observed upon starting the console, after loading a new show file, or if the console's operating mode was recently
-         changed.</t>
   </si>
   <si>
     <t xml:space="preserve"> The console is not in the correct operating mode (e.g., not in playback mode), or an 'override' or 'clear all' command has not been properly executed, leaving the console in a non-control state.</t>
@@ -345,32 +310,16 @@
     <t>Lighting Console Lacks Control While Lights Are On</t>
   </si>
   <si>
-    <t>Despite lighting fixtures being visibly illuminated, the lighting console fails to adjust their intensity, color, or other parameters
-         when faders are moved or cues are activated.</t>
-  </si>
-  <si>
     <t>Typically occurs after a system power cycle, or if a keypad preset has been activated that overrides console control.</t>
   </si>
   <si>
-    <t>A pre-programmed lighting scene or a DMX input from another source (like a keypad) is overriding the console's output, or the
-         console is not properly patched to the fixtures.</t>
-  </si>
-  <si>
     <t>KB0011</t>
   </si>
   <si>
     <t>ProPresenter Lighting Macros Not Triggering Console</t>
   </si>
   <si>
-    <t>Executing a lighting macro within ProPresenter (CUMU-G002) does not result in the expected lighting changes on the console
-         (ZLKU-C001).</t>
-  </si>
-  <si>
     <t>Observed when attempting to fire pre-programmed lighting cues from ProPresenter by clicking the associated macro.</t>
-  </si>
-  <si>
-    <t>The lighting automation software   (e.g., running on CUMU-G001) responsible for translating
-         ProPresenter commands to the lighting console is either not running or has crashed.</t>
   </si>
   <si>
     <t>1) Easiest way to fix this is to logoff CUMU-G001 and logon again.
@@ -395,15 +344,7 @@
     <t>ProPresenter Audio Not Reaching Audio Console (Dante)</t>
   </si>
   <si>
-    <t>Despite active audio meters within ProPresenter (CUMU-G002) during playback, no audio signal is received by the main audio console or
-         other Dante-enabled devices.</t>
-  </si>
-  <si>
     <t>Occurs upon system startup, after a reboot of CUMU-G002, or if Dante connectivity was recently interrupted.</t>
-  </si>
-  <si>
-    <t>The Dante Virtual Soundcard (DVS) application on CUMU-G002 is either not running or not correctly configured, preventing audio
-         routing to the Dante network.</t>
   </si>
   <si>
     <t>1) on CUMU-G002, start the program Dante Virtual Soundcard.
@@ -423,10 +364,6 @@
   </si>
   <si>
     <t>Reaper (Livestream) Not Receiving Audio Input (Dante)</t>
-  </si>
-  <si>
-    <t>Audio is present and audible in the Front of House (FoH) system, but the Reaper DAW on the livestream computer (CUMU-E001) shows no
-         incoming audio signal or active meters.</t>
   </si>
   <si>
     <t>Typically observed after the livestream computer (CUMU-E001) startup, or if Dante connectivity has been interrupted.</t>
@@ -490,9 +427,6 @@
   </si>
   <si>
     <t>System hung</t>
-  </si>
-  <si>
-    <t>power cycle the ZVKU-A001 device using the power button on the rear.</t>
   </si>
   <si>
     <t>#ZVKU-A001</t>
@@ -1043,10 +977,6 @@
   </si>
   <si>
     <t>Waking CUMU-G002 from sleep or booting up when the KVM switch is slow to initialize.</t>
-  </si>
-  <si>
-    <t>KVM switch latency causes the OS to identify the secondary projection output as the primary
-     display, placing the login dialog on a screen not visible to the operator.</t>
   </si>
   <si>
     <t xml:space="preserve">1. Remote login via ScreenConnect or Screen Sharing (from CUMU-G001 go to System Settings &gt; Displays &gt; Arrange, and drag the white menu bar to the local monitor. OR 
@@ -1615,6 +1545,60 @@
   </si>
   <si>
     <t>#propresenter, #keyboard</t>
+  </si>
+  <si>
+    <t>Executing a lighting macro within ProPresenter (CUMU-G002) does not result in the expected lighting changes on the console (ZLKU-C001).</t>
+  </si>
+  <si>
+    <t>The lighting automation software   (e.g., running on CUMU-G001) responsible for translating ProPresenter commands to the lighting console is either not running or has crashed.</t>
+  </si>
+  <si>
+    <t>The Dante Virtual Soundcard (DVS) application on CUMU-G002 is either not running or not correctly configured, preventing audio routing to the Dante network.</t>
+  </si>
+  <si>
+    <t>Despite active audio meters within ProPresenter (CUMU-G002) during playback, no audio signal is received by the main audio console or other Dante-enabled devices.</t>
+  </si>
+  <si>
+    <t>You need to be pretty much directly below each projection screen and point the remote at the projector.  One remote will do all three but you will have to change the selector switch for each projector (not sure if the switch is labelled 1,2,3 or A,B,C.) The east screen is the "first" ( A or 1).</t>
+  </si>
+  <si>
+    <t>Occurs sporadically after system startup, or if the Web Presenter's USB connection to the computer (CUMU-G001) is disturbed.</t>
+  </si>
+  <si>
+    <t>The USB driver for the Web Presenter on CUMU-G001 has become unresponsive, or the USB connection has momentarily dropped, requiring a reset of the USB device to re-establish communication.</t>
+  </si>
+  <si>
+    <t>Upon activating the 'Key 1 Cut' in ATEM Software Control or pressing the 'Lyrics' button on the Stream Deck, the ProPresenter lyric overlay fails to appear on the program output.</t>
+  </si>
+  <si>
+    <t>Observed when attempting to display lyric overlays after an ATEM software update, system reconfiguration, or if keyer settings were manually adjusted.</t>
+  </si>
+  <si>
+    <t>Incorrect or altered 'Key 1' DSK (Downstream Keyer) settings within the ATEM software, specifically the 'Fill Source', 'Key Source', or 'Key Type' parameters, preventing the overlay from rendering correctly.</t>
+  </si>
+  <si>
+    <t>Misalignment or obstruction within the blind's track system, excessive tension on the fabric, or a mechanical issue with the motor or winding mechanism causing it to dislodge.</t>
+  </si>
+  <si>
+    <t>A motorized blackout blind is visibly out of its side track, causing it to be stuck during movement or fail to fully seal against the window frame.</t>
+  </si>
+  <si>
+    <t>Observed upon starting the console, after loading a new show file, or if the console's operating mode was recently changed.</t>
+  </si>
+  <si>
+    <t>A pre-programmed lighting scene or a DMX input from another source (like a keypad) is overriding the console's output, or the console is not properly patched to the fixtures.</t>
+  </si>
+  <si>
+    <t>Despite lighting fixtures being visibly illuminated, the lighting console fails to adjust their intensity, color, or other parameters when faders are moved or cues are activated.</t>
+  </si>
+  <si>
+    <t>Audio is present and audible in the Front of House (FoH) system, but the Reaper DAW on the livestream computer (CUMU-E001) shows no  incoming audio signal or active meters.</t>
+  </si>
+  <si>
+    <t>Power cycle the ZVKU-A001 device using the power button on the rear.</t>
+  </si>
+  <si>
+    <t>KVM switch latency causes the OS to identify the secondary projection output as the primary display, placing the login dialog on a screen not visible to the operator.</t>
   </si>
 </sst>
 </file>
@@ -2246,7 +2230,7 @@
         <v>25</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>436</v>
+        <v>418</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>26</v>
@@ -2292,19 +2276,19 @@
         <v>36</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>432</v>
+        <v>414</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>435</v>
+        <v>417</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="J4" s="4" t="s">
         <v>37</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>438</v>
+        <v>420</v>
       </c>
       <c r="L4" s="4"/>
       <c r="M4" s="4">
@@ -2340,16 +2324,16 @@
         <v>44</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>45</v>
+        <v>470</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>28</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>446</v>
+        <v>428</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="L5" s="4"/>
       <c r="M5" s="4">
@@ -2362,7 +2346,7 @@
     </row>
     <row r="6" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>22</v>
@@ -2371,22 +2355,22 @@
         <v>33</v>
       </c>
       <c r="D6" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E6" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="F6" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="G6" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="H6" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="H6" s="4" t="s">
-        <v>52</v>
-      </c>
       <c r="I6" s="4" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="J6" s="4" t="s">
         <v>37</v>
@@ -2395,7 +2379,7 @@
         <v>38</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>428</v>
+        <v>410</v>
       </c>
       <c r="M6" s="4">
         <v>4</v>
@@ -2407,37 +2391,37 @@
     </row>
     <row r="7" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>22</v>
       </c>
       <c r="C7" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="E7" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="F7" s="4" t="s">
+        <v>471</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="H7" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="I7" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="J7" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="G7" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>317</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>60</v>
-      </c>
       <c r="K7" s="4" t="s">
-        <v>439</v>
+        <v>421</v>
       </c>
       <c r="L7" s="4"/>
       <c r="M7" s="4">
@@ -2450,7 +2434,7 @@
     </row>
     <row r="8" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>22</v>
@@ -2459,28 +2443,28 @@
         <v>33</v>
       </c>
       <c r="D8" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G8" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="H8" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="I8" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="J8" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="G8" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>67</v>
-      </c>
       <c r="K8" s="4" t="s">
-        <v>425</v>
+        <v>407</v>
       </c>
       <c r="L8" s="4"/>
       <c r="M8" s="4">
@@ -2493,7 +2477,7 @@
     </row>
     <row r="9" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>22</v>
@@ -2502,28 +2486,28 @@
         <v>33</v>
       </c>
       <c r="D9" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>473</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>474</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="K9" s="4" t="s">
         <v>69</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="K9" s="4" t="s">
-        <v>75</v>
       </c>
       <c r="L9" s="4"/>
       <c r="M9" s="4">
@@ -2536,35 +2520,35 @@
     </row>
     <row r="10" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>80</v>
+        <v>477</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>82</v>
+        <v>476</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>426</v>
+        <v>408</v>
       </c>
       <c r="J10" s="4"/>
       <c r="K10" s="4" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4">
@@ -2577,37 +2561,37 @@
     </row>
     <row r="11" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>89</v>
+        <v>478</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>93</v>
+        <v>84</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4">
@@ -2620,37 +2604,37 @@
     </row>
     <row r="12" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C12" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D12" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>95</v>
-      </c>
       <c r="E12" s="4" t="s">
-        <v>96</v>
+        <v>480</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>98</v>
+        <v>479</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>437</v>
+        <v>419</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>93</v>
+        <v>84</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4">
@@ -2663,37 +2647,37 @@
     </row>
     <row r="13" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>101</v>
+        <v>466</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>103</v>
+        <v>467</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4">
@@ -2706,40 +2690,40 @@
     </row>
     <row r="14" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>110</v>
+        <v>97</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>111</v>
+        <v>469</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>112</v>
+        <v>98</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>113</v>
+        <v>468</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>114</v>
+        <v>99</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="L14" s="4" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="M14" s="4">
         <v>13</v>
@@ -2751,40 +2735,40 @@
     </row>
     <row r="15" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="B15" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>481</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="J15" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="I15" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="J15" s="4" t="s">
-        <v>124</v>
-      </c>
       <c r="K15" s="4" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
       <c r="L15" s="4" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="M15" s="4">
         <v>14</v>
@@ -2796,7 +2780,7 @@
     </row>
     <row r="16" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
-        <v>126</v>
+        <v>110</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>22</v>
@@ -2805,28 +2789,28 @@
         <v>33</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>128</v>
+        <v>112</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>129</v>
+        <v>113</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>130</v>
+        <v>114</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>131</v>
+        <v>115</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>132</v>
+        <v>116</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4">
@@ -2836,45 +2820,45 @@
         <v>31</v>
       </c>
       <c r="O16" s="4" t="s">
-        <v>134</v>
+        <v>118</v>
       </c>
     </row>
     <row r="17" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
-        <v>135</v>
+        <v>119</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>22</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>136</v>
+        <v>120</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>137</v>
+        <v>121</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>138</v>
+        <v>122</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>139</v>
+        <v>123</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>140</v>
+        <v>124</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>141</v>
+        <v>482</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>142</v>
+        <v>125</v>
       </c>
       <c r="K17" s="4" t="s">
-        <v>143</v>
+        <v>126</v>
       </c>
       <c r="L17" s="6" t="s">
-        <v>471</v>
+        <v>453</v>
       </c>
       <c r="M17" s="4">
         <v>16</v>
@@ -2886,37 +2870,37 @@
     </row>
     <row r="18" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
-        <v>144</v>
+        <v>127</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>22</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>145</v>
+        <v>128</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>146</v>
+        <v>129</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>147</v>
+        <v>130</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>148</v>
+        <v>131</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>149</v>
+        <v>132</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>150</v>
+        <v>133</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="J18" s="4" t="s">
-        <v>151</v>
+        <v>134</v>
       </c>
       <c r="K18" s="4" t="s">
-        <v>152</v>
+        <v>135</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="4">
@@ -2929,37 +2913,37 @@
     </row>
     <row r="19" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
-        <v>153</v>
+        <v>136</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>154</v>
+        <v>137</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>155</v>
+        <v>138</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>156</v>
+        <v>139</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>157</v>
+        <v>140</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>158</v>
+        <v>141</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>159</v>
+        <v>142</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="J19" s="4" t="s">
-        <v>160</v>
+        <v>143</v>
       </c>
       <c r="K19" s="4" t="s">
-        <v>161</v>
+        <v>144</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4">
@@ -2972,37 +2956,37 @@
     </row>
     <row r="20" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
-        <v>162</v>
+        <v>145</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>163</v>
+        <v>146</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>164</v>
+        <v>147</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>165</v>
+        <v>148</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>166</v>
+        <v>149</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>167</v>
+        <v>150</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="J20" s="4" t="s">
-        <v>168</v>
+        <v>151</v>
       </c>
       <c r="K20" s="4" t="s">
-        <v>169</v>
+        <v>152</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4">
@@ -3015,37 +2999,37 @@
     </row>
     <row r="21" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
-        <v>170</v>
+        <v>153</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>171</v>
+        <v>154</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>172</v>
+        <v>155</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>173</v>
+        <v>156</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>174</v>
+        <v>157</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>175</v>
+        <v>158</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>176</v>
+        <v>159</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="J21" s="4" t="s">
-        <v>177</v>
+        <v>160</v>
       </c>
       <c r="K21" s="4" t="s">
-        <v>178</v>
+        <v>161</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4">
@@ -3055,42 +3039,42 @@
         <v>31</v>
       </c>
       <c r="O21" s="4" t="s">
-        <v>179</v>
+        <v>162</v>
       </c>
     </row>
     <row r="22" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
-        <v>180</v>
+        <v>163</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>181</v>
+        <v>164</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>182</v>
+        <v>165</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>184</v>
+        <v>167</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>185</v>
+        <v>168</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>186</v>
+        <v>169</v>
       </c>
       <c r="I22" s="4" t="s">
-        <v>187</v>
+        <v>170</v>
       </c>
       <c r="J22" s="4" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="K22" s="4" t="s">
-        <v>188</v>
+        <v>171</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4">
@@ -3100,42 +3084,42 @@
         <v>31</v>
       </c>
       <c r="O22" s="4" t="s">
-        <v>189</v>
+        <v>172</v>
       </c>
     </row>
     <row r="23" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
-        <v>190</v>
+        <v>173</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>191</v>
+        <v>174</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>192</v>
+        <v>175</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>193</v>
+        <v>176</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>194</v>
+        <v>177</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>195</v>
+        <v>178</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>196</v>
+        <v>179</v>
       </c>
       <c r="I23" s="4" t="s">
-        <v>197</v>
+        <v>180</v>
       </c>
       <c r="J23" s="4" t="s">
-        <v>198</v>
+        <v>181</v>
       </c>
       <c r="K23" s="4" t="s">
-        <v>199</v>
+        <v>182</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4">
@@ -3145,42 +3129,42 @@
         <v>31</v>
       </c>
       <c r="O23" s="4" t="s">
-        <v>200</v>
+        <v>183</v>
       </c>
     </row>
     <row r="24" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
-        <v>201</v>
+        <v>184</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>202</v>
+        <v>185</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>203</v>
+        <v>186</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>204</v>
+        <v>187</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>205</v>
+        <v>188</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>206</v>
+        <v>189</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>207</v>
+        <v>190</v>
       </c>
       <c r="I24" s="4" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="J24" s="4" t="s">
-        <v>208</v>
+        <v>191</v>
       </c>
       <c r="K24" s="4" t="s">
-        <v>209</v>
+        <v>192</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4">
@@ -3190,40 +3174,40 @@
         <v>31</v>
       </c>
       <c r="O24" s="4" t="s">
-        <v>210</v>
+        <v>193</v>
       </c>
     </row>
     <row r="25" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
-        <v>211</v>
+        <v>194</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>212</v>
+        <v>195</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>213</v>
+        <v>196</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>214</v>
+        <v>197</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>215</v>
+        <v>198</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>216</v>
+        <v>199</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>433</v>
+        <v>415</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="J25" s="4"/>
       <c r="K25" s="4" t="s">
-        <v>217</v>
+        <v>200</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4">
@@ -3236,7 +3220,7 @@
     </row>
     <row r="26" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
-        <v>430</v>
+        <v>412</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>16</v>
@@ -3261,7 +3245,7 @@
     </row>
     <row r="27" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
-        <v>218</v>
+        <v>201</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>22</v>
@@ -3270,28 +3254,28 @@
         <v>23</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>219</v>
+        <v>202</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>220</v>
+        <v>203</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>221</v>
+        <v>204</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>222</v>
+        <v>205</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>223</v>
+        <v>206</v>
       </c>
       <c r="I27" s="4" t="s">
         <v>22</v>
       </c>
       <c r="J27" s="4" t="s">
-        <v>224</v>
+        <v>207</v>
       </c>
       <c r="K27" s="4" t="s">
-        <v>225</v>
+        <v>208</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4">
@@ -3301,87 +3285,87 @@
         <v>31</v>
       </c>
       <c r="O27" s="4" t="s">
-        <v>226</v>
+        <v>209</v>
       </c>
     </row>
     <row r="28" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
-        <v>227</v>
+        <v>210</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>228</v>
+        <v>211</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>229</v>
+        <v>212</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>230</v>
+        <v>213</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>231</v>
+        <v>214</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>232</v>
+        <v>215</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>233</v>
+        <v>216</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>434</v>
+        <v>416</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>234</v>
+        <v>217</v>
       </c>
       <c r="J28" s="4" t="s">
-        <v>235</v>
+        <v>218</v>
       </c>
       <c r="K28" s="4" t="s">
-        <v>236</v>
+        <v>219</v>
       </c>
       <c r="L28" s="4"/>
       <c r="M28" s="4">
         <v>26</v>
       </c>
       <c r="N28" s="4" t="s">
-        <v>237</v>
+        <v>220</v>
       </c>
       <c r="O28" s="4" t="s">
-        <v>238</v>
+        <v>221</v>
       </c>
     </row>
     <row r="29" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
-        <v>239</v>
+        <v>222</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>240</v>
+        <v>223</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>241</v>
+        <v>224</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>242</v>
+        <v>225</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>243</v>
+        <v>226</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>244</v>
+        <v>227</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="J29" s="4" t="s">
-        <v>245</v>
+        <v>228</v>
       </c>
       <c r="K29" s="4" t="s">
-        <v>246</v>
+        <v>229</v>
       </c>
       <c r="L29" s="4"/>
       <c r="M29" s="4">
@@ -3391,42 +3375,42 @@
         <v>31</v>
       </c>
       <c r="O29" s="4" t="s">
-        <v>247</v>
+        <v>230</v>
       </c>
     </row>
     <row r="30" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
-        <v>248</v>
+        <v>231</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>249</v>
+        <v>232</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>250</v>
+        <v>233</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>251</v>
+        <v>234</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>252</v>
+        <v>235</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>253</v>
+        <v>236</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>254</v>
+        <v>237</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="J30" s="4" t="s">
-        <v>427</v>
+        <v>409</v>
       </c>
       <c r="K30" s="4" t="s">
-        <v>255</v>
+        <v>238</v>
       </c>
       <c r="L30" s="4"/>
       <c r="M30" s="4">
@@ -3436,42 +3420,42 @@
         <v>31</v>
       </c>
       <c r="O30" s="4" t="s">
-        <v>256</v>
+        <v>239</v>
       </c>
     </row>
     <row r="31" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
-        <v>257</v>
+        <v>240</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>22</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>258</v>
+        <v>241</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>259</v>
+        <v>242</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>260</v>
+        <v>243</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>261</v>
+        <v>244</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>262</v>
+        <v>245</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>263</v>
+        <v>246</v>
       </c>
       <c r="I31" s="4" t="s">
         <v>22</v>
       </c>
       <c r="J31" s="4" t="s">
-        <v>298</v>
+        <v>281</v>
       </c>
       <c r="K31" s="4" t="s">
-        <v>264</v>
+        <v>247</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4">
@@ -3481,42 +3465,42 @@
         <v>31</v>
       </c>
       <c r="O31" s="4" t="s">
-        <v>265</v>
+        <v>248</v>
       </c>
     </row>
     <row r="32" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
-        <v>266</v>
+        <v>249</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>267</v>
+        <v>250</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>268</v>
+        <v>251</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>269</v>
+        <v>252</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>270</v>
+        <v>253</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>271</v>
+        <v>254</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>272</v>
+        <v>255</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="J32" s="4" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="K32" s="4" t="s">
-        <v>273</v>
+        <v>256</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4">
@@ -3526,40 +3510,40 @@
         <v>31</v>
       </c>
       <c r="O32" s="4" t="s">
-        <v>274</v>
+        <v>257</v>
       </c>
     </row>
     <row r="33" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
-        <v>275</v>
+        <v>258</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>276</v>
+        <v>259</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>277</v>
+        <v>260</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>278</v>
+        <v>261</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>279</v>
+        <v>262</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>280</v>
+        <v>263</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>281</v>
+        <v>264</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>282</v>
+        <v>265</v>
       </c>
       <c r="I33" s="4" t="s">
-        <v>277</v>
+        <v>260</v>
       </c>
       <c r="J33" s="4"/>
       <c r="K33" s="4" t="s">
-        <v>283</v>
+        <v>266</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4">
@@ -3569,42 +3553,42 @@
         <v>31</v>
       </c>
       <c r="O33" s="4" t="s">
-        <v>284</v>
+        <v>267</v>
       </c>
     </row>
     <row r="34" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
-        <v>285</v>
+        <v>268</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>286</v>
+        <v>269</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>287</v>
+        <v>270</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>288</v>
+        <v>271</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>289</v>
+        <v>272</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>429</v>
+        <v>411</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="J34" s="4" t="s">
-        <v>245</v>
+        <v>228</v>
       </c>
       <c r="K34" s="4" t="s">
-        <v>290</v>
+        <v>273</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4">
@@ -3614,42 +3598,42 @@
         <v>31</v>
       </c>
       <c r="O34" s="4" t="s">
-        <v>291</v>
+        <v>274</v>
       </c>
     </row>
     <row r="35" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
-        <v>431</v>
+        <v>413</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>22</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>317</v>
+        <v>299</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>440</v>
+        <v>422</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>441</v>
+        <v>423</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>442</v>
+        <v>424</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>443</v>
+        <v>425</v>
       </c>
       <c r="H35" s="4" t="s">
-        <v>444</v>
+        <v>426</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>317</v>
+        <v>299</v>
       </c>
       <c r="J35" s="4" t="s">
-        <v>307</v>
+        <v>289</v>
       </c>
       <c r="K35" s="4" t="s">
-        <v>445</v>
+        <v>427</v>
       </c>
       <c r="L35" s="4"/>
       <c r="M35" s="4">
@@ -3662,37 +3646,37 @@
     </row>
     <row r="36" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
-        <v>292</v>
+        <v>275</v>
       </c>
       <c r="B36" s="4" t="s">
         <v>22</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>293</v>
+        <v>276</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>294</v>
+        <v>277</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>295</v>
+        <v>278</v>
       </c>
       <c r="G36" s="4" t="s">
-        <v>296</v>
+        <v>279</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>297</v>
+        <v>280</v>
       </c>
       <c r="I36" s="4" t="s">
         <v>22</v>
       </c>
       <c r="J36" s="4" t="s">
-        <v>298</v>
+        <v>281</v>
       </c>
       <c r="K36" s="4" t="s">
-        <v>299</v>
+        <v>282</v>
       </c>
       <c r="L36" s="4"/>
       <c r="M36" s="4">
@@ -3702,42 +3686,42 @@
         <v>31</v>
       </c>
       <c r="O36" s="4" t="s">
-        <v>300</v>
+        <v>283</v>
       </c>
     </row>
     <row r="37" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
-        <v>301</v>
+        <v>284</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>22</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>302</v>
+        <v>285</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>303</v>
+        <v>286</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>304</v>
+        <v>287</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>305</v>
+        <v>483</v>
       </c>
       <c r="H37" s="4" t="s">
-        <v>306</v>
+        <v>288</v>
       </c>
       <c r="I37" s="4" t="s">
         <v>22</v>
       </c>
       <c r="J37" s="4" t="s">
-        <v>307</v>
+        <v>289</v>
       </c>
       <c r="K37" s="4" t="s">
-        <v>308</v>
+        <v>290</v>
       </c>
       <c r="L37" s="4"/>
       <c r="M37" s="4">
@@ -3747,45 +3731,45 @@
         <v>31</v>
       </c>
       <c r="O37" s="4" t="s">
-        <v>309</v>
+        <v>291</v>
       </c>
     </row>
     <row r="38" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
-        <v>310</v>
+        <v>292</v>
       </c>
       <c r="B38" s="4" t="s">
         <v>22</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>311</v>
+        <v>293</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>312</v>
+        <v>294</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>313</v>
+        <v>295</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>314</v>
+        <v>296</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>315</v>
+        <v>297</v>
       </c>
       <c r="H38" s="4" t="s">
-        <v>316</v>
+        <v>298</v>
       </c>
       <c r="I38" s="4" t="s">
-        <v>424</v>
+        <v>406</v>
       </c>
       <c r="J38" s="4" t="s">
         <v>37</v>
       </c>
       <c r="K38" s="4" t="s">
-        <v>318</v>
+        <v>300</v>
       </c>
       <c r="L38" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="M38" s="4">
         <v>36</v>
@@ -3794,42 +3778,42 @@
         <v>31</v>
       </c>
       <c r="O38" s="4" t="s">
-        <v>319</v>
+        <v>301</v>
       </c>
     </row>
     <row r="39" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
-        <v>320</v>
+        <v>302</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>22</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>311</v>
+        <v>293</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>321</v>
+        <v>303</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>322</v>
+        <v>304</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>323</v>
+        <v>305</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>324</v>
+        <v>306</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>422</v>
+        <v>404</v>
       </c>
       <c r="I39" s="4" t="s">
-        <v>317</v>
+        <v>299</v>
       </c>
       <c r="J39" s="4" t="s">
-        <v>423</v>
+        <v>405</v>
       </c>
       <c r="K39" s="4" t="s">
-        <v>325</v>
+        <v>307</v>
       </c>
       <c r="L39" s="4"/>
       <c r="M39" s="4">
@@ -3839,42 +3823,42 @@
         <v>31</v>
       </c>
       <c r="O39" s="4" t="s">
-        <v>421</v>
+        <v>403</v>
       </c>
     </row>
     <row r="40" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
-        <v>455</v>
+        <v>437</v>
       </c>
       <c r="B40" s="4" t="s">
         <v>22</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>447</v>
+        <v>429</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>448</v>
+        <v>430</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>449</v>
+        <v>431</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>450</v>
+        <v>432</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>451</v>
+        <v>433</v>
       </c>
       <c r="I40" s="4" t="s">
-        <v>317</v>
+        <v>299</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>452</v>
+        <v>434</v>
       </c>
       <c r="K40" s="4" t="s">
-        <v>453</v>
+        <v>435</v>
       </c>
       <c r="L40" s="4"/>
       <c r="M40" s="4">
@@ -3884,12 +3868,12 @@
         <v>31</v>
       </c>
       <c r="O40" s="4" t="s">
-        <v>454</v>
+        <v>436</v>
       </c>
     </row>
     <row r="41" spans="1:15" s="5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
-        <v>456</v>
+        <v>438</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>22</v>
@@ -3898,28 +3882,28 @@
         <v>23</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>457</v>
+        <v>439</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>458</v>
+        <v>440</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>459</v>
+        <v>441</v>
       </c>
       <c r="G41" s="4" t="s">
-        <v>460</v>
+        <v>442</v>
       </c>
       <c r="H41" s="4" t="s">
-        <v>461</v>
+        <v>443</v>
       </c>
       <c r="I41" s="4" t="s">
         <v>28</v>
       </c>
       <c r="J41" s="4" t="s">
-        <v>462</v>
+        <v>444</v>
       </c>
       <c r="K41" s="4" t="s">
-        <v>463</v>
+        <v>445</v>
       </c>
       <c r="L41" s="4"/>
       <c r="M41" s="4">
@@ -3932,33 +3916,33 @@
     </row>
     <row r="42" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
-        <v>464</v>
+        <v>446</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>277</v>
+        <v>260</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>277</v>
+        <v>260</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>465</v>
+        <v>447</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>466</v>
+        <v>448</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>467</v>
+        <v>449</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>468</v>
+        <v>450</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>469</v>
+        <v>451</v>
       </c>
       <c r="I42" s="4"/>
       <c r="J42" s="4"/>
       <c r="K42" s="4" t="s">
-        <v>283</v>
+        <v>266</v>
       </c>
       <c r="L42" s="4"/>
       <c r="M42" s="4">
@@ -3968,45 +3952,45 @@
         <v>31</v>
       </c>
       <c r="O42" s="4" t="s">
-        <v>470</v>
+        <v>452</v>
       </c>
     </row>
     <row r="43" spans="1:15" ht="51" x14ac:dyDescent="0.2">
       <c r="A43" s="6" t="s">
-        <v>471</v>
+        <v>453</v>
       </c>
       <c r="B43" s="7" t="s">
         <v>22</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>472</v>
+        <v>454</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>473</v>
+        <v>455</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>474</v>
+        <v>456</v>
       </c>
       <c r="G43" s="7" t="s">
-        <v>140</v>
+        <v>124</v>
       </c>
       <c r="H43" s="7" t="s">
-        <v>141</v>
+        <v>482</v>
       </c>
       <c r="I43" s="7" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="J43" s="7" t="s">
-        <v>142</v>
+        <v>125</v>
       </c>
       <c r="K43" s="7" t="s">
-        <v>143</v>
+        <v>126</v>
       </c>
       <c r="L43" s="7" t="s">
-        <v>135</v>
+        <v>119</v>
       </c>
       <c r="M43" s="7">
         <v>44</v>
@@ -4015,45 +3999,45 @@
         <v>31</v>
       </c>
       <c r="O43" s="8" t="s">
-        <v>475</v>
+        <v>457</v>
       </c>
     </row>
     <row r="44" spans="1:15" ht="51" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
-        <v>476</v>
+        <v>458</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>22</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>477</v>
+        <v>459</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>478</v>
+        <v>460</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>479</v>
+        <v>461</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>480</v>
+        <v>462</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>481</v>
+        <v>463</v>
       </c>
       <c r="I44" s="4" t="s">
-        <v>317</v>
+        <v>299</v>
       </c>
       <c r="J44" s="4" t="s">
-        <v>482</v>
+        <v>464</v>
       </c>
       <c r="K44" s="4" t="s">
-        <v>483</v>
+        <v>465</v>
       </c>
       <c r="L44" s="4" t="s">
-        <v>455</v>
+        <v>437</v>
       </c>
       <c r="M44" s="4">
         <v>45</v>
@@ -4078,477 +4062,477 @@
   <sheetData>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>326</v>
+        <v>308</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>327</v>
+        <v>309</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>328</v>
+        <v>310</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>329</v>
+        <v>311</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>330</v>
+        <v>312</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>331</v>
+        <v>313</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>332</v>
+        <v>314</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>333</v>
+        <v>315</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>334</v>
+        <v>316</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>335</v>
+        <v>317</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>336</v>
+        <v>318</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>337</v>
+        <v>319</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>338</v>
+        <v>320</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>339</v>
+        <v>321</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>340</v>
+        <v>322</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>341</v>
+        <v>323</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>342</v>
+        <v>324</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>343</v>
+        <v>325</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>344</v>
+        <v>326</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>345</v>
+        <v>327</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>346</v>
+        <v>328</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>347</v>
+        <v>329</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>348</v>
+        <v>330</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>349</v>
+        <v>331</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>350</v>
+        <v>332</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>351</v>
+        <v>333</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>352</v>
+        <v>334</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>353</v>
+        <v>335</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>354</v>
+        <v>336</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>355</v>
+        <v>337</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>356</v>
+        <v>338</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>357</v>
+        <v>339</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>358</v>
+        <v>340</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>359</v>
+        <v>341</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>360</v>
+        <v>342</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>361</v>
+        <v>343</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>362</v>
+        <v>344</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>363</v>
+        <v>345</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>364</v>
+        <v>346</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>365</v>
+        <v>347</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>366</v>
+        <v>348</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>367</v>
+        <v>349</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>368</v>
+        <v>350</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>369</v>
+        <v>351</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>370</v>
+        <v>352</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>371</v>
+        <v>353</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>372</v>
+        <v>354</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>373</v>
+        <v>355</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>374</v>
+        <v>356</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>375</v>
+        <v>357</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>376</v>
+        <v>358</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>377</v>
+        <v>359</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>378</v>
+        <v>360</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>379</v>
+        <v>361</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>380</v>
+        <v>362</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>381</v>
+        <v>363</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>382</v>
+        <v>364</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>383</v>
+        <v>365</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>384</v>
+        <v>366</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>385</v>
+        <v>367</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>386</v>
+        <v>368</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>387</v>
+        <v>369</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>388</v>
+        <v>370</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>389</v>
+        <v>371</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>390</v>
+        <v>372</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A82" s="2" t="s">
-        <v>391</v>
+        <v>373</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A85" s="3" t="s">
-        <v>392</v>
+        <v>374</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A86" s="3" t="s">
-        <v>393</v>
+        <v>375</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A87" s="3" t="s">
-        <v>394</v>
+        <v>376</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A88" s="3" t="s">
-        <v>395</v>
+        <v>377</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A89" s="3" t="s">
-        <v>396</v>
+        <v>378</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A90" s="3" t="s">
-        <v>397</v>
+        <v>379</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A91" s="3" t="s">
-        <v>398</v>
+        <v>380</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A94" s="3" t="s">
-        <v>399</v>
+        <v>381</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A95" s="3" t="s">
-        <v>400</v>
+        <v>382</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A96" s="3" t="s">
-        <v>401</v>
+        <v>383</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A97" s="3" t="s">
-        <v>402</v>
+        <v>384</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A98" s="3" t="s">
-        <v>403</v>
+        <v>385</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A99" s="3" t="s">
-        <v>404</v>
+        <v>386</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A100" s="3" t="s">
-        <v>405</v>
+        <v>387</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A103" s="3" t="s">
-        <v>406</v>
+        <v>388</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A104" s="3" t="s">
-        <v>407</v>
+        <v>389</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A105" s="3" t="s">
-        <v>408</v>
+        <v>390</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A106" s="3" t="s">
-        <v>409</v>
+        <v>391</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A107" s="3" t="s">
-        <v>410</v>
+        <v>392</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A108" s="3" t="s">
-        <v>411</v>
+        <v>393</v>
       </c>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A109" s="3" t="s">
-        <v>412</v>
+        <v>394</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A112" s="3" t="s">
-        <v>413</v>
+        <v>395</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A113" s="3" t="s">
-        <v>414</v>
+        <v>396</v>
       </c>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A114" s="3" t="s">
-        <v>415</v>
+        <v>397</v>
       </c>
     </row>
     <row r="115" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A115" s="3" t="s">
-        <v>416</v>
+        <v>398</v>
       </c>
     </row>
     <row r="116" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A116" s="3" t="s">
-        <v>417</v>
+        <v>399</v>
       </c>
     </row>
     <row r="117" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A117" s="3" t="s">
-        <v>418</v>
+        <v>400</v>
       </c>
     </row>
     <row r="118" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A118" s="3" t="s">
-        <v>419</v>
+        <v>401</v>
       </c>
     </row>
     <row r="119" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A119" s="3" t="s">
-        <v>420</v>
+        <v>402</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
corrections/additions post power failure event
</commit_message>
<xml_diff>
--- a/knowledgebase.xlsx
+++ b/knowledgebase.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D5AC2AC-0AE7-B549-B84B-71C4A97FF96D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AFEAF3B-3DAD-DC4A-B91A-5BA7BEDF4C85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="661" uniqueCount="501">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="696" uniqueCount="526">
   <si>
     <t xml:space="preserve"> IssueID </t>
   </si>
@@ -1654,6 +1654,85 @@
     <t>1) check connections
 2) Reboot CUMU-G001
 3) As a fallback, use the buttons that are on the front face of the video mixer in the rack. You can view the multiview display on the video hub 2507-0700 monitor .</t>
+  </si>
+  <si>
+    <t>KB0046</t>
+  </si>
+  <si>
+    <t>Lights don't respond even though console is powered on and operating.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Firing a Cue, or manually setting a look doesn't result in a lighting change. </t>
+  </si>
+  <si>
+    <t>There is an overriding control that is preventing the lights from repsonding.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) If exepcting on of the cues to first, make sure that the executor master fader for the sequence is at 100% ( usually the first fader). 
+2) The "Blind" or  "Prvw" buttons might be active. They are in the centre of the console. They are lit when active. Press them to turn them off. </t>
+  </si>
+  <si>
+    <t>Lighting, Control</t>
+  </si>
+  <si>
+    <t>2507-2500</t>
+  </si>
+  <si>
+    <t>#lighting, #control</t>
+  </si>
+  <si>
+    <t>KB0047</t>
+  </si>
+  <si>
+    <t>Montior does not respond</t>
+  </si>
+  <si>
+    <t>Unsure of what can cause this. It happened once after a major power failure.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cause not determined. </t>
+  </si>
+  <si>
+    <t>Computer, Video</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) try selecting inputs hdmi1 and hdmi2. 
+2) Verify that the computer is on (indicator light is on)
+3) try logging in from another computer either using MacOS screen sharing or the remote access solution. If you can than that indicates the problem is with the video subsystem and not the computer itself.
+4) open the rack (2602-1800) side panels to locate the decimator (ZVIU-C001), there is a red hdmi cable (2310-1004) plugged into that device.  Unplug it and replug. </t>
+  </si>
+  <si>
+    <t>CUMU-G002, 2311-2701, ZVIU-C001, 2310-1004</t>
+  </si>
+  <si>
+    <t>Despite the monitor (2311-2701) being powered on and hdmi 1 or 2 are selected, the display remains black.</t>
+  </si>
+  <si>
+    <t>KB0048</t>
+  </si>
+  <si>
+    <t>Audio system does not power up despite the touch panel appearing to behave normally.</t>
+  </si>
+  <si>
+    <t>Pressing the Power button on the touch screeen intiates the normal power up animations, but the system does not actually power on. The gear beside the surface does not power up, nor does the surface itself, nor the amplifiers in the main rack.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This has been observed after a major power outage that outlasted the UPS reserve. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loss of system power left the control system in a confused state. </t>
+  </si>
+  <si>
+    <t>From one of the media arts Mac computers, login to the website http://192.168.200.50/.  You will get a warning about the website not being private. This is acceptable. Click Show details, and then "visit this website" - message text could be slightly different depening on which browser you are using. Navigate to "utilities" on the left hand side, and then select "Reboot" beside "Core Reboot". It will take a few minutes to complete. Then try the touch screen again.</t>
+  </si>
+  <si>
+    <t>2408-2704, 2407-3001</t>
+  </si>
+  <si>
+    <t>#audio, #power</t>
+  </si>
+  <si>
+    <t>#video, #monitor</t>
   </si>
 </sst>
 </file>
@@ -1838,8 +1917,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8DA13CB4-8680-0D4C-A016-6564C2E20834}" name="Table1" displayName="Table1" ref="A1:O46" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
-  <autoFilter ref="A1:O46" xr:uid="{8DA13CB4-8680-0D4C-A016-6564C2E20834}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8DA13CB4-8680-0D4C-A016-6564C2E20834}" name="Table1" displayName="Table1" ref="A1:O49" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
+  <autoFilter ref="A1:O49" xr:uid="{8DA13CB4-8680-0D4C-A016-6564C2E20834}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:O40">
     <sortCondition ref="A2:A40"/>
   </sortState>
@@ -2181,7 +2260,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O46"/>
+  <dimension ref="A1:O49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.5" style="1" customWidth="1"/>
@@ -4201,6 +4280,133 @@
       </c>
       <c r="O46" s="4"/>
     </row>
+    <row r="47" spans="1:15" ht="187" x14ac:dyDescent="0.2">
+      <c r="A47" s="4" t="s">
+        <v>501</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>503</v>
+      </c>
+      <c r="F47" s="4"/>
+      <c r="G47" s="4" t="s">
+        <v>504</v>
+      </c>
+      <c r="H47" s="4" t="s">
+        <v>505</v>
+      </c>
+      <c r="I47" s="4" t="s">
+        <v>506</v>
+      </c>
+      <c r="J47" s="4" t="s">
+        <v>507</v>
+      </c>
+      <c r="K47" s="4" t="s">
+        <v>508</v>
+      </c>
+      <c r="L47" s="4"/>
+      <c r="M47" s="4">
+        <v>47</v>
+      </c>
+      <c r="N47" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="O47" s="4"/>
+    </row>
+    <row r="48" spans="1:15" ht="306" x14ac:dyDescent="0.2">
+      <c r="A48" s="4" t="s">
+        <v>509</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>510</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>516</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>511</v>
+      </c>
+      <c r="G48" s="4" t="s">
+        <v>512</v>
+      </c>
+      <c r="H48" s="4" t="s">
+        <v>514</v>
+      </c>
+      <c r="I48" s="4" t="s">
+        <v>513</v>
+      </c>
+      <c r="J48" s="4" t="s">
+        <v>515</v>
+      </c>
+      <c r="K48" s="4" t="s">
+        <v>525</v>
+      </c>
+      <c r="L48" s="4"/>
+      <c r="M48" s="4">
+        <v>47</v>
+      </c>
+      <c r="N48" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="O48" s="4"/>
+    </row>
+    <row r="49" spans="1:15" ht="289" x14ac:dyDescent="0.2">
+      <c r="A49" s="4" t="s">
+        <v>517</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>518</v>
+      </c>
+      <c r="E49" s="4" t="s">
+        <v>519</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>520</v>
+      </c>
+      <c r="G49" s="4" t="s">
+        <v>521</v>
+      </c>
+      <c r="H49" s="4" t="s">
+        <v>522</v>
+      </c>
+      <c r="I49" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="J49" s="4" t="s">
+        <v>523</v>
+      </c>
+      <c r="K49" s="4" t="s">
+        <v>524</v>
+      </c>
+      <c r="L49" s="4"/>
+      <c r="M49" s="4">
+        <v>48</v>
+      </c>
+      <c r="N49" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="O49" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Updated a few items
</commit_message>
<xml_diff>
--- a/knowledgebase.xlsx
+++ b/knowledgebase.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AFEAF3B-3DAD-DC4A-B91A-5BA7BEDF4C85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EB160F4-9690-8041-8F03-9B0414B3CCB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20" yWindow="660" windowWidth="30240" windowHeight="13660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Issues" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="696" uniqueCount="526">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="526">
   <si>
     <t xml:space="preserve"> IssueID </t>
   </si>
@@ -972,16 +972,7 @@
     <t>Presenter Login Dialog Missing on Local Monitor</t>
   </si>
   <si>
-    <t>Local monitor shows only the desktop background/wallpaper with no login fields, icons, or
-     interactive elements.</t>
-  </si>
-  <si>
     <t>Waking CUMU-G002 from sleep or booting up when the KVM switch is slow to initialize.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Remote login via ScreenConnect or Screen Sharing (from CUMU-G001 go to System Settings &gt; Displays &gt; Arrange, and drag the white menu bar to the local monitor. OR 
-2. Route the "PPHD" source to the ATEM Program/Preview monitor to see and interact with the dialog. OR 
-3. (Hardware  Fix) Unplug cable 2308-0918 from the rear of CUMU-G002 to force the OS to use the local monitor. </t>
   </si>
   <si>
     <t>CUMU-G002</t>
@@ -1668,10 +1659,6 @@
     <t>There is an overriding control that is preventing the lights from repsonding.</t>
   </si>
   <si>
-    <t xml:space="preserve">1) If exepcting on of the cues to first, make sure that the executor master fader for the sequence is at 100% ( usually the first fader). 
-2) The "Blind" or  "Prvw" buttons might be active. They are in the centre of the console. They are lit when active. Press them to turn them off. </t>
-  </si>
-  <si>
     <t>Lighting, Control</t>
   </si>
   <si>
@@ -1733,6 +1720,20 @@
   </si>
   <si>
     <t>#video, #monitor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) If exepcting on of the cues to first, make sure that the executor master fader for the sequence is at 100% ( usually the first fader). 
+2) The "Blind" or  "Prvw" buttons might be active. If they are in the centre of the console. They are lit when active. Press them to turn them off. </t>
+  </si>
+  <si>
+    <t>Local monitor shows only the desktop background/wallpaper with no login fields, icons, or interactive elements.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Try each of these in order:
+1. On the stream deck, select "Main Menu", then "Video Menu", then "VIdeo Hub".  There are now two buttons at the bottom "PP Operator 1" and "PP Operator 2". Press each in turn until you see the login prompt.
+2. Remote login via ScreenConnect or Screen Sharing (from CUMU-G001 go to System Settings &gt; Displays &gt; Arrange, and drag the white menu bar to the local monitor. OR 
+3. Route the "PPHD" source to the ATEM Program/Preview monitor to see and interact with the dialog. OR 
+4. (Hardware  Fix) Unplug cable 2308-0918 from the rear of CUMU-G002 to force the OS to use the local monitor. </t>
   </si>
 </sst>
 </file>
@@ -2371,7 +2372,7 @@
         <v>25</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>26</v>
@@ -2417,10 +2418,10 @@
         <v>36</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="I4" s="4" t="s">
         <v>68</v>
@@ -2429,7 +2430,7 @@
         <v>37</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="L4" s="4"/>
       <c r="M4" s="4">
@@ -2465,13 +2466,13 @@
         <v>44</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>28</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="K5" s="4" t="s">
         <v>45</v>
@@ -2520,7 +2521,7 @@
         <v>38</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="M6" s="4">
         <v>4</v>
@@ -2547,22 +2548,22 @@
         <v>55</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>56</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="J7" s="4" t="s">
         <v>57</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="L7" s="4"/>
       <c r="M7" s="4">
@@ -2605,7 +2606,7 @@
         <v>64</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="L8" s="4"/>
       <c r="M8" s="4">
@@ -2630,13 +2631,13 @@
         <v>66</v>
       </c>
       <c r="E9" s="4" t="s">
+        <v>470</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>471</v>
+      </c>
+      <c r="G9" s="4" t="s">
         <v>472</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>473</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>474</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>67</v>
@@ -2673,19 +2674,19 @@
         <v>73</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="F10" s="4" t="s">
         <v>74</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>75</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="J10" s="4"/>
       <c r="K10" s="4" t="s">
@@ -2717,7 +2718,7 @@
         <v>80</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="G11" s="4" t="s">
         <v>81</v>
@@ -2757,16 +2758,16 @@
         <v>86</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="F12" s="4" t="s">
         <v>87</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="I12" s="4" t="s">
         <v>68</v>
@@ -2800,13 +2801,13 @@
         <v>89</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>90</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="H13" s="4" t="s">
         <v>91</v>
@@ -2820,7 +2821,9 @@
       <c r="K13" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="L13" s="4"/>
+      <c r="L13" s="4" t="s">
+        <v>499</v>
+      </c>
       <c r="M13" s="4">
         <v>12</v>
       </c>
@@ -2843,13 +2846,13 @@
         <v>97</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="F14" s="4" t="s">
         <v>98</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="H14" s="4" t="s">
         <v>99</v>
@@ -2888,7 +2891,7 @@
         <v>104</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="F15" s="4" t="s">
         <v>105</v>
@@ -2987,7 +2990,7 @@
         <v>124</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="I17" s="4" t="s">
         <v>68</v>
@@ -2999,7 +3002,7 @@
         <v>126</v>
       </c>
       <c r="L17" s="6" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="M17" s="4">
         <v>16</v>
@@ -3341,7 +3344,7 @@
         <v>199</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="I25" s="4" t="s">
         <v>95</v>
@@ -3361,7 +3364,7 @@
     </row>
     <row r="26" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>16</v>
@@ -3452,7 +3455,7 @@
         <v>216</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="I28" s="4" t="s">
         <v>217</v>
@@ -3548,7 +3551,7 @@
         <v>95</v>
       </c>
       <c r="J30" s="4" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="K30" s="4" t="s">
         <v>238</v>
@@ -3720,7 +3723,7 @@
         <v>272</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="I34" s="4" t="s">
         <v>68</v>
@@ -3744,37 +3747,37 @@
     </row>
     <row r="35" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>22</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="D35" s="4" t="s">
+        <v>420</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>421</v>
+      </c>
+      <c r="F35" s="4" t="s">
         <v>422</v>
       </c>
-      <c r="E35" s="4" t="s">
+      <c r="G35" s="4" t="s">
         <v>423</v>
       </c>
-      <c r="F35" s="4" t="s">
+      <c r="H35" s="4" t="s">
         <v>424</v>
       </c>
-      <c r="G35" s="4" t="s">
+      <c r="I35" s="4" t="s">
+        <v>297</v>
+      </c>
+      <c r="J35" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="K35" s="4" t="s">
         <v>425</v>
-      </c>
-      <c r="H35" s="4" t="s">
-        <v>426</v>
-      </c>
-      <c r="I35" s="4" t="s">
-        <v>299</v>
-      </c>
-      <c r="J35" s="4" t="s">
-        <v>289</v>
-      </c>
-      <c r="K35" s="4" t="s">
-        <v>427</v>
       </c>
       <c r="L35" s="4"/>
       <c r="M35" s="4">
@@ -3830,7 +3833,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="37" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:15" s="5" customFormat="1" ht="263" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
         <v>284</v>
       </c>
@@ -3844,25 +3847,25 @@
         <v>285</v>
       </c>
       <c r="E37" s="4" t="s">
+        <v>524</v>
+      </c>
+      <c r="F37" s="4" t="s">
         <v>286</v>
       </c>
-      <c r="F37" s="4" t="s">
-        <v>287</v>
-      </c>
       <c r="G37" s="4" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="H37" s="4" t="s">
-        <v>288</v>
+        <v>525</v>
       </c>
       <c r="I37" s="4" t="s">
         <v>22</v>
       </c>
       <c r="J37" s="4" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="K37" s="4" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="L37" s="4"/>
       <c r="M37" s="4">
@@ -3872,42 +3875,42 @@
         <v>31</v>
       </c>
       <c r="O37" s="4" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="38" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="B38" s="4" t="s">
         <v>22</v>
       </c>
       <c r="C38" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>292</v>
+      </c>
+      <c r="E38" s="4" t="s">
         <v>293</v>
       </c>
-      <c r="D38" s="4" t="s">
+      <c r="F38" s="4" t="s">
         <v>294</v>
       </c>
-      <c r="E38" s="4" t="s">
+      <c r="G38" s="4" t="s">
         <v>295</v>
       </c>
-      <c r="F38" s="4" t="s">
+      <c r="H38" s="4" t="s">
         <v>296</v>
       </c>
-      <c r="G38" s="4" t="s">
-        <v>297</v>
-      </c>
-      <c r="H38" s="4" t="s">
-        <v>298</v>
-      </c>
       <c r="I38" s="4" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="J38" s="4" t="s">
         <v>37</v>
       </c>
       <c r="K38" s="4" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="L38" s="4" t="s">
         <v>46</v>
@@ -3919,42 +3922,42 @@
         <v>31</v>
       </c>
       <c r="O38" s="4" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="39" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>22</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="D39" s="4" t="s">
+        <v>301</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="F39" s="4" t="s">
         <v>303</v>
       </c>
-      <c r="E39" s="4" t="s">
+      <c r="G39" s="4" t="s">
         <v>304</v>
       </c>
-      <c r="F39" s="4" t="s">
+      <c r="H39" s="4" t="s">
+        <v>402</v>
+      </c>
+      <c r="I39" s="4" t="s">
+        <v>297</v>
+      </c>
+      <c r="J39" s="4" t="s">
+        <v>403</v>
+      </c>
+      <c r="K39" s="4" t="s">
         <v>305</v>
-      </c>
-      <c r="G39" s="4" t="s">
-        <v>306</v>
-      </c>
-      <c r="H39" s="4" t="s">
-        <v>404</v>
-      </c>
-      <c r="I39" s="4" t="s">
-        <v>299</v>
-      </c>
-      <c r="J39" s="4" t="s">
-        <v>405</v>
-      </c>
-      <c r="K39" s="4" t="s">
-        <v>307</v>
       </c>
       <c r="L39" s="4"/>
       <c r="M39" s="4">
@@ -3964,12 +3967,12 @@
         <v>31</v>
       </c>
       <c r="O39" s="4" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="40" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="B40" s="4" t="s">
         <v>22</v>
@@ -3978,28 +3981,28 @@
         <v>96</v>
       </c>
       <c r="D40" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="F40" s="4" t="s">
         <v>429</v>
       </c>
-      <c r="E40" s="4" t="s">
+      <c r="G40" s="4" t="s">
         <v>430</v>
       </c>
-      <c r="F40" s="4" t="s">
+      <c r="H40" s="4" t="s">
         <v>431</v>
       </c>
-      <c r="G40" s="4" t="s">
+      <c r="I40" s="4" t="s">
+        <v>297</v>
+      </c>
+      <c r="J40" s="4" t="s">
         <v>432</v>
       </c>
-      <c r="H40" s="4" t="s">
+      <c r="K40" s="4" t="s">
         <v>433</v>
-      </c>
-      <c r="I40" s="4" t="s">
-        <v>299</v>
-      </c>
-      <c r="J40" s="4" t="s">
-        <v>434</v>
-      </c>
-      <c r="K40" s="4" t="s">
-        <v>435</v>
       </c>
       <c r="L40" s="4"/>
       <c r="M40" s="4">
@@ -4009,12 +4012,12 @@
         <v>31</v>
       </c>
       <c r="O40" s="4" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
     </row>
     <row r="41" spans="1:15" s="5" customFormat="1" ht="68" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>22</v>
@@ -4023,28 +4026,28 @@
         <v>23</v>
       </c>
       <c r="D41" s="4" t="s">
+        <v>437</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>490</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="G41" s="4" t="s">
         <v>439</v>
       </c>
-      <c r="E41" s="4" t="s">
-        <v>492</v>
-      </c>
-      <c r="F41" s="4" t="s">
+      <c r="H41" s="4" t="s">
         <v>440</v>
-      </c>
-      <c r="G41" s="4" t="s">
-        <v>441</v>
-      </c>
-      <c r="H41" s="4" t="s">
-        <v>442</v>
       </c>
       <c r="I41" s="4" t="s">
         <v>28</v>
       </c>
       <c r="J41" s="4" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="K41" s="4" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="L41" s="4"/>
       <c r="M41" s="4">
@@ -4054,12 +4057,12 @@
         <v>31</v>
       </c>
       <c r="O41" s="4" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
     </row>
     <row r="42" spans="1:15" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>260</v>
@@ -4068,19 +4071,19 @@
         <v>260</v>
       </c>
       <c r="D42" s="4" t="s">
+        <v>444</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="F42" s="4" t="s">
         <v>446</v>
       </c>
-      <c r="E42" s="4" t="s">
+      <c r="G42" s="4" t="s">
         <v>447</v>
       </c>
-      <c r="F42" s="4" t="s">
+      <c r="H42" s="4" t="s">
         <v>448</v>
-      </c>
-      <c r="G42" s="4" t="s">
-        <v>449</v>
-      </c>
-      <c r="H42" s="4" t="s">
-        <v>450</v>
       </c>
       <c r="I42" s="4"/>
       <c r="J42" s="4"/>
@@ -4095,12 +4098,12 @@
         <v>31</v>
       </c>
       <c r="O42" s="4" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
     </row>
     <row r="43" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="6" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="B43" s="7" t="s">
         <v>22</v>
@@ -4109,19 +4112,19 @@
         <v>68</v>
       </c>
       <c r="D43" s="7" t="s">
+        <v>451</v>
+      </c>
+      <c r="E43" s="7" t="s">
+        <v>452</v>
+      </c>
+      <c r="F43" s="7" t="s">
         <v>453</v>
-      </c>
-      <c r="E43" s="7" t="s">
-        <v>454</v>
-      </c>
-      <c r="F43" s="7" t="s">
-        <v>455</v>
       </c>
       <c r="G43" s="7" t="s">
         <v>124</v>
       </c>
       <c r="H43" s="7" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="I43" s="7" t="s">
         <v>68</v>
@@ -4142,12 +4145,12 @@
         <v>31</v>
       </c>
       <c r="O43" s="8" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
     </row>
     <row r="44" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>22</v>
@@ -4156,31 +4159,31 @@
         <v>96</v>
       </c>
       <c r="D44" s="4" t="s">
+        <v>456</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>457</v>
+      </c>
+      <c r="F44" s="4" t="s">
         <v>458</v>
       </c>
-      <c r="E44" s="4" t="s">
+      <c r="G44" s="4" t="s">
         <v>459</v>
       </c>
-      <c r="F44" s="4" t="s">
+      <c r="H44" s="4" t="s">
         <v>460</v>
       </c>
-      <c r="G44" s="4" t="s">
+      <c r="I44" s="4" t="s">
+        <v>297</v>
+      </c>
+      <c r="J44" s="4" t="s">
         <v>461</v>
       </c>
-      <c r="H44" s="4" t="s">
+      <c r="K44" s="4" t="s">
         <v>462</v>
       </c>
-      <c r="I44" s="4" t="s">
-        <v>299</v>
-      </c>
-      <c r="J44" s="4" t="s">
-        <v>463</v>
-      </c>
-      <c r="K44" s="4" t="s">
-        <v>464</v>
-      </c>
       <c r="L44" s="4" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="M44" s="4">
         <v>45</v>
@@ -4192,7 +4195,7 @@
     </row>
     <row r="45" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="4" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="B45" s="4" t="s">
         <v>22</v>
@@ -4201,28 +4204,28 @@
         <v>96</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="E45" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>481</v>
+      </c>
+      <c r="G45" s="4" t="s">
+        <v>483</v>
+      </c>
+      <c r="H45" s="4" t="s">
         <v>484</v>
       </c>
-      <c r="F45" s="4" t="s">
-        <v>483</v>
-      </c>
-      <c r="G45" s="4" t="s">
+      <c r="I45" s="4" t="s">
         <v>485</v>
       </c>
-      <c r="H45" s="4" t="s">
+      <c r="J45" s="4" t="s">
         <v>486</v>
       </c>
-      <c r="I45" s="4" t="s">
-        <v>487</v>
-      </c>
-      <c r="J45" s="4" t="s">
-        <v>488</v>
-      </c>
       <c r="K45" s="4" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="L45" s="4" t="s">
         <v>284</v>
@@ -4234,12 +4237,12 @@
         <v>31</v>
       </c>
       <c r="O45" s="4" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
     </row>
     <row r="46" spans="1:15" ht="136" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="B46" s="4" t="s">
         <v>22</v>
@@ -4248,29 +4251,29 @@
         <v>241</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="F46" s="4"/>
       <c r="G46" s="4" t="s">
+        <v>495</v>
+      </c>
+      <c r="H46" s="4" t="s">
+        <v>498</v>
+      </c>
+      <c r="I46" s="4" t="s">
+        <v>485</v>
+      </c>
+      <c r="J46" s="4" t="s">
+        <v>496</v>
+      </c>
+      <c r="K46" s="4" t="s">
         <v>497</v>
       </c>
-      <c r="H46" s="4" t="s">
-        <v>500</v>
-      </c>
-      <c r="I46" s="4" t="s">
+      <c r="L46" s="4" t="s">
         <v>487</v>
-      </c>
-      <c r="J46" s="4" t="s">
-        <v>498</v>
-      </c>
-      <c r="K46" s="4" t="s">
-        <v>499</v>
-      </c>
-      <c r="L46" s="4" t="s">
-        <v>489</v>
       </c>
       <c r="M46" s="4">
         <v>46</v>
@@ -4282,7 +4285,7 @@
     </row>
     <row r="47" spans="1:15" ht="187" x14ac:dyDescent="0.2">
       <c r="A47" s="4" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="B47" s="4" t="s">
         <v>71</v>
@@ -4291,28 +4294,30 @@
         <v>78</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="F47" s="4"/>
       <c r="G47" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="H47" s="4" t="s">
+        <v>523</v>
+      </c>
+      <c r="I47" s="4" t="s">
+        <v>503</v>
+      </c>
+      <c r="J47" s="4" t="s">
         <v>504</v>
       </c>
-      <c r="H47" s="4" t="s">
+      <c r="K47" s="4" t="s">
         <v>505</v>
       </c>
-      <c r="I47" s="4" t="s">
-        <v>506</v>
-      </c>
-      <c r="J47" s="4" t="s">
-        <v>507</v>
-      </c>
-      <c r="K47" s="4" t="s">
-        <v>508</v>
-      </c>
-      <c r="L47" s="4"/>
+      <c r="L47" s="4" t="s">
+        <v>88</v>
+      </c>
       <c r="M47" s="4">
         <v>47</v>
       </c>
@@ -4323,7 +4328,7 @@
     </row>
     <row r="48" spans="1:15" ht="306" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="B48" s="4" t="s">
         <v>22</v>
@@ -4332,28 +4337,28 @@
         <v>96</v>
       </c>
       <c r="D48" s="4" t="s">
+        <v>507</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>513</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>508</v>
+      </c>
+      <c r="G48" s="4" t="s">
+        <v>509</v>
+      </c>
+      <c r="H48" s="4" t="s">
+        <v>511</v>
+      </c>
+      <c r="I48" s="4" t="s">
         <v>510</v>
       </c>
-      <c r="E48" s="4" t="s">
-        <v>516</v>
-      </c>
-      <c r="F48" s="4" t="s">
-        <v>511</v>
-      </c>
-      <c r="G48" s="4" t="s">
+      <c r="J48" s="4" t="s">
         <v>512</v>
       </c>
-      <c r="H48" s="4" t="s">
-        <v>514</v>
-      </c>
-      <c r="I48" s="4" t="s">
-        <v>513</v>
-      </c>
-      <c r="J48" s="4" t="s">
-        <v>515</v>
-      </c>
       <c r="K48" s="4" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="L48" s="4"/>
       <c r="M48" s="4">
@@ -4364,9 +4369,9 @@
       </c>
       <c r="O48" s="4"/>
     </row>
-    <row r="49" spans="1:15" ht="289" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:15" ht="68" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="B49" s="4" t="s">
         <v>95</v>
@@ -4375,28 +4380,28 @@
         <v>68</v>
       </c>
       <c r="D49" s="4" t="s">
+        <v>515</v>
+      </c>
+      <c r="E49" s="4" t="s">
+        <v>516</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>517</v>
+      </c>
+      <c r="G49" s="4" t="s">
         <v>518</v>
       </c>
-      <c r="E49" s="4" t="s">
+      <c r="H49" s="4" t="s">
         <v>519</v>
-      </c>
-      <c r="F49" s="4" t="s">
-        <v>520</v>
-      </c>
-      <c r="G49" s="4" t="s">
-        <v>521</v>
-      </c>
-      <c r="H49" s="4" t="s">
-        <v>522</v>
       </c>
       <c r="I49" s="4" t="s">
         <v>68</v>
       </c>
       <c r="J49" s="4" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="K49" s="4" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="L49" s="4"/>
       <c r="M49" s="4">
@@ -4422,477 +4427,477 @@
   <sheetData>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A82" s="2" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A85" s="3" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A86" s="3" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A87" s="3" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A88" s="3" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A89" s="3" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A90" s="3" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A91" s="3" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A94" s="3" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A95" s="3" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A96" s="3" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A97" s="3" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A98" s="3" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A99" s="3" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A100" s="3" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A103" s="3" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A104" s="3" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A105" s="3" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A106" s="3" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A107" s="3" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A108" s="3" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A109" s="3" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A112" s="3" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A113" s="3" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A114" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="115" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A115" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="116" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A116" s="3" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="117" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A117" s="3" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="118" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A118" s="3" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="119" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A119" s="3" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added dante resolution failed item
</commit_message>
<xml_diff>
--- a/knowledgebase.xlsx
+++ b/knowledgebase.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EC9CC24-1279-A342-BF61-A21FF5F76DA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{341CE5BD-3C0E-F449-81F9-D9345DDCFC93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="660" windowWidth="30240" windowHeight="13660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Issues" sheetId="1" r:id="rId1"/>
     <sheet name="Metadata" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="526">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="741" uniqueCount="540">
   <si>
     <t xml:space="preserve"> IssueID </t>
   </si>
@@ -1735,12 +1736,75 @@
 3. Route the "PPHD" source to the ATEM Program/Preview monitor to see and interact with the dialog,  go to System Settings &gt; Displays &gt; Arrange, and drag the white menu bar to the local monitor. OR 
 4. (Hardware  Fix) Unplug cable 2308-0918 from the rear of CUMU-G002 to force the OS to use the local monitor. </t>
   </si>
+  <si>
+    <t xml:space="preserve">Reaper periodically goes silent for a few seconds. </t>
+  </si>
+  <si>
+    <t>During livestream operation, all audio inputs go silent, for perhaps 3 seconds, and then it returns to normal operation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">With Dante Controller running, wait for the event to recur. Dante Controller's event log shows an error "Resolution Failed" for CUMU-E001. </t>
+  </si>
+  <si>
+    <t>Root cause unknown.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> If still in rehearsal (ie not actively broadcasting):
+1) Reboot CUMU-E001.
+If broadcasting: 
+1) Set the house dlive console's video matrix to mirror the FOH audio, but at elevated levels.This could be done on the physical surface (2407-3001) or via dlive director (2607-2321).
+2) Using the Q-SYS touchpad (2408-2704) or the app on CUMU-E001, switch video source to 'Matrix'. 
+3) Reboot CUMU-E001 and re-establish the Reaper session.
+4) Using the Q-SYS touchpad (2408-2704) or the app on CUMU-E001, switch video source to 'DAW'.
+If sitation continues to occur, consider switching the video source to Matrix. You can actively mix the inputs using the matrix mix on dlive director.  </t>
+  </si>
+  <si>
+    <t>Audio, Computer</t>
+  </si>
+  <si>
+    <t>CUMU-E001, 2607-2302, 2607-2306</t>
+  </si>
+  <si>
+    <t>#audio, #dante</t>
+  </si>
+  <si>
+    <t>This has only happened once.</t>
+  </si>
+  <si>
+    <t>KB0049</t>
+  </si>
+  <si>
+    <t>Root cause unknown. The Dante 'Resolution Failed' error for CUMU-E001 in the event log points to a Dante device-discovery/name-resolution dropout rather than a Reaper fault.</t>
+  </si>
+  <si>
+    <t>This has only happened once; during rehearsal on 2026-08-23.</t>
+  </si>
+  <si>
+    <t>With Dante Controller running, wait for the event to recur. Dante Controller's event log shows an error "Resolution Failed" for CUMU-E001. 
+If the event recurs, capture diagnostics before rebooting (the reboot clears the event state):
+In Dante Controller, navigate to the 'Events' tab and use the 'Save' button at the bottom to capture the event diagnostics for later review.
+While in the 'Events' tab, check whether the errors are logged only against CUMU-E001 or against multiple devices. Errors on CUMU-E001 alone suggest a fault local to that node; errors across several devices suggest a wider Dante network problem (switch, clock/PTP, or cabling).
+In the device list, note whether CUMU-E001 briefly disappears at the moment of the dropout, or stays present but drops its subscriptions. Disappearing points to a discovery/name-resolution fault; staying present with lost subscriptions points to a subscription/flow fault.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note: Video' matrix and 'Video Send' selector are named for the video broadcast they feed, but both carry audio. Normal operation for broadcasting runs with 'Video Send' set to 'DAW'
+If still in rehearsal (ie not actively broadcasting):
+1) Capture diagnostics per TriggerConditions (save the Events log and note single-node vs. system-wide).
+2) Reboot CUMU-E001.
+If broadcasting:
+1) Set the house dlive console's 'Video' matrix (the backup audio mix for the broadcast) to mirror the FOH audio, but at elevated levels. This can be done on the physical surface (2407-3001) or via dlive director (2607-2321).
+2) Using the Q-SYS touchpad (2408-2704) or the app on CUMU-E001, set 'Video Send' to 'Matrix'.
+3) Capture diagnostics per TriggerConditions (save the Events log and note single-node vs. system-wide, before rebooting).
+4) Reboot CUMU-E001 and re-establish the Reaper session.
+5) Using the Q-SYS touchpad (2408-2704) or the app on CUMU-E001, set 'Video Send' back to 'DAW'."
+If situation continues to occur, consider switching the video source to Matrix. You can actively mix the inputs using the matrix mix on dlive director.  </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1768,16 +1832,36 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor theme="6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor theme="6" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -1822,11 +1906,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="6" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="6" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="6" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="6" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="6" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="6" tint="0.39997558519241921"/>
+      </right>
+      <top style="thin">
+        <color theme="6" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="6" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1846,6 +1967,24 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1918,8 +2057,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8DA13CB4-8680-0D4C-A016-6564C2E20834}" name="Table1" displayName="Table1" ref="A1:O49" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
-  <autoFilter ref="A1:O49" xr:uid="{8DA13CB4-8680-0D4C-A016-6564C2E20834}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8DA13CB4-8680-0D4C-A016-6564C2E20834}" name="Table1" displayName="Table1" ref="A1:O50" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
+  <autoFilter ref="A1:O50" xr:uid="{8DA13CB4-8680-0D4C-A016-6564C2E20834}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:O40">
     <sortCondition ref="A2:A40"/>
   </sortState>
@@ -2261,7 +2400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O49"/>
+  <dimension ref="A1:O50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.5" style="1" customWidth="1"/>
@@ -4412,6 +4551,53 @@
       </c>
       <c r="O49" s="4"/>
     </row>
+    <row r="50" spans="1:15" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A50" s="4" t="s">
+        <v>535</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>526</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>527</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>538</v>
+      </c>
+      <c r="G50" s="4" t="s">
+        <v>536</v>
+      </c>
+      <c r="H50" s="4" t="s">
+        <v>539</v>
+      </c>
+      <c r="I50" s="4" t="s">
+        <v>531</v>
+      </c>
+      <c r="J50" s="4" t="s">
+        <v>532</v>
+      </c>
+      <c r="K50" s="4" t="s">
+        <v>533</v>
+      </c>
+      <c r="L50" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="M50" s="4">
+        <v>50</v>
+      </c>
+      <c r="N50" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="O50" s="4" t="s">
+        <v>537</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -4903,4 +5089,138 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D34FA1E-DACB-4A40-A2D8-391D868E6BDF}">
+  <dimension ref="A2:B16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="15.1640625" customWidth="1"/>
+    <col min="2" max="2" width="137.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A2" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A3" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="51" x14ac:dyDescent="0.2">
+      <c r="A4" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="85" x14ac:dyDescent="0.2">
+      <c r="A5" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="204" x14ac:dyDescent="0.2">
+      <c r="A6" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="255" x14ac:dyDescent="0.2">
+      <c r="A7" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="51" x14ac:dyDescent="0.2">
+      <c r="A8" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A9" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="51" x14ac:dyDescent="0.2">
+      <c r="A10" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="68" x14ac:dyDescent="0.2">
+      <c r="A11" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="34" x14ac:dyDescent="0.2">
+      <c r="A12" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A13" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A14" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="13">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A15" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="68" x14ac:dyDescent="0.2">
+      <c r="A16" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>534</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>